<commit_message>
fix: updated static xlsx file
</commit_message>
<xml_diff>
--- a/static/МСБ Свод (общий).xlsx
+++ b/static/МСБ Свод (общий).xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_BS1">Лист1!$C:$C</definedName>
-    <definedName name="_INTERNAL_KEY1">Лист1!$4:$4</definedName>
+    <definedName name="_INTERNAL_KEY1">Лист1!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
 </workbook>
@@ -47,7 +47,7 @@
     <author>tc={008A0083-00DF-450A-8D5D-0075004A00C9}</author>
   </authors>
   <commentList>
-    <comment ref="B15" authorId="0" shapeId="0">
+    <comment ref="B16" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -64,7 +64,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B16" authorId="1" shapeId="0">
+    <comment ref="B17" authorId="1" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -81,7 +81,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B18" authorId="2" shapeId="0">
+    <comment ref="B19" authorId="2" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -98,7 +98,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B21" authorId="3" shapeId="0">
+    <comment ref="B22" authorId="3" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -115,7 +115,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B26" authorId="4" shapeId="0">
+    <comment ref="B27" authorId="4" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -132,7 +132,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B27" authorId="5" shapeId="0">
+    <comment ref="B28" authorId="5" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -149,7 +149,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B35" authorId="6" shapeId="0">
+    <comment ref="B36" authorId="6" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -166,7 +166,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A41" authorId="7" shapeId="0">
+    <comment ref="A42" authorId="7" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -183,7 +183,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B44" authorId="8" shapeId="0">
+    <comment ref="B45" authorId="8" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -200,7 +200,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B46" authorId="9" shapeId="0">
+    <comment ref="B47" authorId="9" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -217,7 +217,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B52" authorId="10" shapeId="0">
+    <comment ref="B53" authorId="10" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -234,7 +234,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B53" authorId="11" shapeId="0">
+    <comment ref="B54" authorId="11" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -251,7 +251,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B55" authorId="12" shapeId="0">
+    <comment ref="B56" authorId="12" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -268,7 +268,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B59" authorId="13" shapeId="0">
+    <comment ref="B60" authorId="13" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -285,7 +285,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B61" authorId="14" shapeId="0">
+    <comment ref="B62" authorId="14" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -304,7 +304,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B62" authorId="15" shapeId="0">
+    <comment ref="B63" authorId="15" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -321,7 +321,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B63" authorId="16" shapeId="0">
+    <comment ref="B64" authorId="16" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -338,7 +338,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B73" authorId="17" shapeId="0">
+    <comment ref="B74" authorId="17" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -355,7 +355,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B77" authorId="18" shapeId="0">
+    <comment ref="B78" authorId="18" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -372,7 +372,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B78" authorId="19" shapeId="0">
+    <comment ref="B79" authorId="19" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1077,7 +1077,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1183,6 +1183,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1200,7 +1215,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1359,48 +1374,55 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="4"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="SAPBEXHLevel0" xfId="2"/>
@@ -1686,7 +1708,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:D80"/>
+  <dimension ref="A2:D81"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
@@ -1696,822 +1718,828 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="63" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="67" t="s">
+      <c r="B2" s="64" t="s">
         <v>181</v>
       </c>
-      <c r="C2" s="60" t="s">
+      <c r="C2" s="71" t="s">
         <v>182</v>
       </c>
-      <c r="D2" s="60" t="s">
+      <c r="D2" s="71" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61"/>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
+      <c r="A3" s="70"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="71"/>
+      <c r="D3" s="71"/>
     </row>
     <row r="4" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="44"/>
-      <c r="B4" s="45"/>
-      <c r="C4" s="46"/>
-    </row>
-    <row r="5" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+      <c r="A4" s="55"/>
+      <c r="B4" s="55"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+    </row>
+    <row r="5" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="44"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="46"/>
+    </row>
+    <row r="6" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
         <v>1</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C6" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D6" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="57" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="65" t="s">
+      <c r="B7" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="36" t="s">
+      <c r="C7" s="36" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="55"/>
-      <c r="B7" s="55"/>
-      <c r="C7" s="36" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="57"/>
+      <c r="B8" s="57"/>
+      <c r="C8" s="36" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="47" t="s">
+    <row r="9" spans="1:4" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="36" t="s">
+      <c r="C9" s="36" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="47"/>
-      <c r="B9" s="5" t="s">
+    <row r="10" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="47"/>
+      <c r="B10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="36" t="s">
+      <c r="C10" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="52" t="s">
+      <c r="D10" s="52" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="47"/>
-      <c r="B10" s="7" t="s">
+    <row r="11" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="47"/>
+      <c r="B11" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="C11" s="37" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+    <row r="12" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="36" t="s">
+      <c r="C12" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D12" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="54" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="67" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="56" t="s">
+      <c r="B13" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="37" t="s">
+      <c r="C13" s="37" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="55"/>
-      <c r="B13" s="55"/>
-      <c r="C13" s="37" t="s">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="57"/>
+      <c r="B14" s="57"/>
+      <c r="C14" s="37" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="48" t="s">
+    <row r="15" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="49" t="s">
+      <c r="B15" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="37" t="s">
+      <c r="C15" s="37" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="47" t="s">
+    <row r="16" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="36" t="s">
+      <c r="C16" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D16" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="57" t="s">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="64" t="s">
+      <c r="B17" s="61" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="38" t="s">
+      <c r="C17" s="38" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="55"/>
-      <c r="B17" s="55"/>
-      <c r="C17" s="36">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="57"/>
+      <c r="B18" s="57"/>
+      <c r="C18" s="36">
         <v>100330143</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="56.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="47" t="s">
+    <row r="19" spans="1:4" ht="56.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B19" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="38" t="s">
+      <c r="C19" s="38" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+    <row r="20" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="50" t="s">
+      <c r="B20" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="36" t="s">
+      <c r="C20" s="36" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="48" t="s">
+    <row r="21" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B21" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="37" t="s">
+      <c r="C21" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D21" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="48" t="s">
+    <row r="22" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B22" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="37" t="s">
+      <c r="C22" s="37" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="48" t="s">
+    <row r="23" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B23" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="37" t="s">
+      <c r="C23" s="37" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="48" t="s">
+    <row r="24" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="48" t="s">
         <v>45</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B24" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="37" t="s">
+      <c r="C24" s="37" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="51"/>
-      <c r="B24" s="13" t="s">
+    <row r="25" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="51"/>
+      <c r="B25" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="39" t="s">
+      <c r="C25" s="39" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6">
+    <row r="26" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="6">
         <v>3</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B26" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="36" t="s">
+      <c r="C26" s="36" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="14" t="s">
+    <row r="27" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B27" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="C26" s="37" t="s">
+      <c r="C27" s="37" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="14" t="s">
+    <row r="28" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="16" t="s">
+      <c r="B28" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C27" s="37" t="s">
+      <c r="C28" s="37" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="4">
+    <row r="29" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="4">
         <v>4</v>
       </c>
-      <c r="B28" s="50" t="s">
+      <c r="B29" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="39" t="s">
+      <c r="C29" s="39" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="57" t="s">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="56" t="s">
         <v>59</v>
       </c>
-      <c r="B29" s="69" t="s">
+      <c r="B30" s="66" t="s">
         <v>60</v>
       </c>
-      <c r="C29" s="36" t="s">
+      <c r="C30" s="36" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="55"/>
-      <c r="B30" s="55"/>
-      <c r="C30" s="36" t="s">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="57"/>
+      <c r="B31" s="57"/>
+      <c r="C31" s="36" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="62" t="s">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="58" t="s">
         <v>63</v>
       </c>
-      <c r="B31" s="68" t="s">
+      <c r="B32" s="65" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="37" t="s">
+      <c r="C32" s="37" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="55"/>
-      <c r="B32" s="55"/>
-      <c r="C32" s="37" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="57"/>
+      <c r="B33" s="57"/>
+      <c r="C33" s="37" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="51" t="s">
+    <row r="34" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="51" t="s">
         <v>67</v>
       </c>
-      <c r="B33" s="58" t="s">
+      <c r="B34" s="69" t="s">
         <v>68</v>
       </c>
-      <c r="C33" s="37" t="s">
+      <c r="C34" s="37" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="51"/>
-      <c r="B34" s="59"/>
-      <c r="C34" s="37" t="s">
+    <row r="35" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="51"/>
+      <c r="B35" s="60"/>
+      <c r="C35" s="37" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="51" t="s">
+    <row r="36" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="51" t="s">
         <v>71</v>
       </c>
-      <c r="B35" s="68" t="s">
+      <c r="B36" s="65" t="s">
         <v>72</v>
       </c>
-      <c r="C35" s="37" t="s">
+      <c r="C36" s="37" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="51"/>
-      <c r="B36" s="55"/>
-      <c r="C36" s="37" t="s">
+    <row r="37" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="51"/>
+      <c r="B37" s="57"/>
+      <c r="C37" s="37" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="47" t="s">
+    <row r="38" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="47" t="s">
         <v>75</v>
       </c>
-      <c r="B37" s="50" t="s">
+      <c r="B38" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="C37" s="36" t="s">
+      <c r="C38" s="36" t="s">
         <v>77</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="B38" s="17" t="s">
-        <v>79</v>
-      </c>
-      <c r="C38" s="37" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="51" t="s">
-        <v>81</v>
-      </c>
-      <c r="B39" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="C39" s="40" t="s">
-        <v>83</v>
+        <v>78</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="C39" s="37" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="51" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C40" s="40" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="51" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C41" s="40" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="51" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C42" s="40" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="51" t="s">
+        <v>90</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C43" s="40" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="51" t="s">
         <v>93</v>
       </c>
-      <c r="B43" s="18" t="s">
+      <c r="B44" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="C43" s="41" t="s">
+      <c r="C44" s="41" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="51"/>
-      <c r="B44" s="13" t="s">
+    <row r="45" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="51"/>
+      <c r="B45" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="C44" s="37" t="s">
+      <c r="C45" s="37" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="51"/>
-      <c r="B45" s="19" t="s">
-        <v>97</v>
-      </c>
-      <c r="C45" s="41" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="51"/>
       <c r="B46" s="19" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C46" s="41" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="51"/>
       <c r="B47" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="C47" s="41" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="51"/>
+      <c r="B48" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C47" s="41" t="s">
+      <c r="C48" s="41" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="47" t="s">
+    <row r="49" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="B48" s="20" t="s">
+      <c r="B49" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="C48" s="42" t="s">
+      <c r="C49" s="42" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="51" t="s">
+    <row r="50" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="51" t="s">
         <v>106</v>
       </c>
-      <c r="B49" s="17" t="s">
+      <c r="B50" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="C49" s="37" t="s">
+      <c r="C50" s="37" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="14"/>
-      <c r="B50" s="21" t="s">
+    <row r="51" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="14"/>
+      <c r="B51" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="C50" s="37" t="s">
+      <c r="C51" s="37" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="22"/>
-      <c r="B51" s="23" t="s">
+    <row r="52" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="22"/>
+      <c r="B52" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="C51" s="37" t="s">
+      <c r="C52" s="37" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="22"/>
-      <c r="B52" s="24" t="s">
+    <row r="53" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="22"/>
+      <c r="B53" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="C52" s="41" t="s">
+      <c r="C53" s="41" t="s">
         <v>113</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="25"/>
-      <c r="B53" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C53" s="41" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="25"/>
-      <c r="B54" s="26" t="s">
+      <c r="B54" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="C54" s="41" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="25"/>
+      <c r="B55" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="C54" s="41" t="s">
+      <c r="C55" s="41" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="22"/>
-      <c r="B55" s="24" t="s">
+    <row r="56" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="22"/>
+      <c r="B56" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="C55" s="41" t="s">
+      <c r="C56" s="41" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="14"/>
-      <c r="B56" s="27" t="s">
+    <row r="57" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="14"/>
+      <c r="B57" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="C56" s="41" t="s">
+      <c r="C57" s="41" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="47" t="s">
+    <row r="58" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="47" t="s">
         <v>120</v>
       </c>
-      <c r="B57" s="50" t="s">
+      <c r="B58" s="50" t="s">
         <v>121</v>
       </c>
-      <c r="C57" s="42" t="s">
+      <c r="C58" s="42" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="47" t="s">
+    <row r="59" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="47" t="s">
         <v>123</v>
       </c>
-      <c r="B58" s="20" t="s">
+      <c r="B59" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="C58" s="42" t="s">
+      <c r="C59" s="42" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="28" t="s">
+    <row r="60" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="28" t="s">
         <v>126</v>
       </c>
-      <c r="B59" s="29" t="s">
+      <c r="B60" s="29" t="s">
         <v>127</v>
       </c>
-      <c r="C59" s="37" t="s">
+      <c r="C60" s="37" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="30"/>
-      <c r="B60" s="23" t="s">
+    <row r="61" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="30"/>
+      <c r="B61" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="C60" s="37" t="s">
+      <c r="C61" s="37" t="s">
         <v>129</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="14"/>
-      <c r="B61" s="16" t="s">
-        <v>130</v>
-      </c>
-      <c r="C61" s="41" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="14"/>
       <c r="B62" s="16" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C62" s="41" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="14"/>
       <c r="B63" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="C63" s="41" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="14"/>
+      <c r="B64" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="C63" s="41" t="s">
+      <c r="C64" s="41" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="47" t="s">
+    <row r="65" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="47" t="s">
         <v>136</v>
       </c>
-      <c r="B64" s="20" t="s">
+      <c r="B65" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="C64" s="36" t="s">
+      <c r="C65" s="36" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="65" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="47"/>
-      <c r="B65" s="31" t="s">
+    <row r="66" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="47"/>
+      <c r="B66" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="C65" s="43" t="s">
+      <c r="C66" s="43" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="66" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="51" t="s">
+    <row r="67" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="51" t="s">
         <v>141</v>
       </c>
-      <c r="B66" s="31" t="s">
+      <c r="B67" s="31" t="s">
         <v>142</v>
       </c>
-      <c r="C66" s="43" t="s">
+      <c r="C67" s="43" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="67" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="51" t="s">
+    <row r="68" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="51" t="s">
         <v>144</v>
       </c>
-      <c r="B67" s="31" t="s">
+      <c r="B68" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="C67" s="43" t="s">
+      <c r="C68" s="43" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="68" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="47" t="s">
+    <row r="69" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="47" t="s">
         <v>147</v>
       </c>
-      <c r="B68" s="20" t="s">
+      <c r="B69" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="C68" s="42" t="s">
+      <c r="C69" s="42" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="47" t="s">
+    <row r="70" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="47" t="s">
         <v>150</v>
       </c>
-      <c r="B69" s="20" t="s">
+      <c r="B70" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="C69" s="42" t="s">
+      <c r="C70" s="42" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="70" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="47" t="s">
+    <row r="71" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="47" t="s">
         <v>153</v>
       </c>
-      <c r="B70" s="20" t="s">
+      <c r="B71" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="C70" s="42" t="s">
+      <c r="C71" s="42" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="71" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="47" t="s">
+    <row r="72" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="47" t="s">
         <v>156</v>
       </c>
-      <c r="B71" s="20" t="s">
+      <c r="B72" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="C71" s="42" t="s">
+      <c r="C72" s="42" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="72" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="47" t="s">
+    <row r="73" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="47" t="s">
         <v>159</v>
       </c>
-      <c r="B72" s="20" t="s">
+      <c r="B73" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="C72" s="42" t="s">
+      <c r="C73" s="42" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="57" t="s">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" s="56" t="s">
         <v>162</v>
       </c>
-      <c r="B73" s="63" t="s">
+      <c r="B74" s="59" t="s">
         <v>163</v>
       </c>
-      <c r="C73" s="42" t="s">
+      <c r="C74" s="42" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="55"/>
-      <c r="B74" s="59"/>
-      <c r="C74" s="36" t="s">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" s="57"/>
+      <c r="B75" s="60"/>
+      <c r="C75" s="36" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="75" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="47" t="s">
+    <row r="76" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A76" s="47" t="s">
         <v>166</v>
       </c>
-      <c r="B75" s="32" t="s">
+      <c r="B76" s="32" t="s">
         <v>167</v>
       </c>
-      <c r="C75" s="39" t="s">
+      <c r="C76" s="39" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="47"/>
-      <c r="B76" s="32" t="s">
+    <row r="77" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A77" s="47"/>
+      <c r="B77" s="32" t="s">
         <v>169</v>
       </c>
-      <c r="C76" s="39" t="s">
+      <c r="C77" s="39" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="47" t="s">
+    <row r="78" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A78" s="47" t="s">
         <v>171</v>
       </c>
-      <c r="B77" s="32" t="s">
+      <c r="B78" s="32" t="s">
         <v>172</v>
       </c>
-      <c r="C77" s="39" t="s">
+      <c r="C78" s="39" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="47"/>
-      <c r="B78" s="23" t="s">
+    <row r="79" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A79" s="47"/>
+      <c r="B79" s="23" t="s">
         <v>174</v>
       </c>
-      <c r="C78" s="36" t="s">
+      <c r="C79" s="36" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="79" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="33"/>
-      <c r="B79" s="34" t="s">
+    <row r="80" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A80" s="33"/>
+      <c r="B80" s="34" t="s">
         <v>176</v>
       </c>
-      <c r="C79" s="36" t="s">
+      <c r="C80" s="36" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C80" s="53" t="s">
+    <row r="81" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C81" s="53" t="s">
         <v>185</v>
       </c>
-      <c r="D80" s="52" t="s">
+      <c r="D81" s="52" t="s">
         <v>184</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="A73:A74"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="A74:A75"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B74:B75"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A7:A8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>